<commit_message>
compact mobile simulation buttons
</commit_message>
<xml_diff>
--- a/public/카드DB.xlsx
+++ b/public/카드DB.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5915" uniqueCount="1111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6605" uniqueCount="1160">
   <si>
     <t>팀</t>
   </si>
@@ -3889,6 +3889,202 @@
   </si>
   <si>
     <t>김태형S</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>박진만</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>장원삼</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>라이블리</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>박충식</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김시진</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>권영호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>피렐라</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>이만수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>박한이</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>최익성</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김진웅</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>탈보트</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>노장진</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>러프</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>배영섭</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>양도근</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김지찬</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>류중일</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>강기웅</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>곽채진</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>임총오</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>오대석</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김무신</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>오봉옥</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>권오준</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>박근홍</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>전병호</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김태한</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>성준</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김한수</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>신동주</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>장태수B</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>허규옥</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김태훈S</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>이승현B</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>최지광</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>김상엽</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>조동찬</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>강봉규</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>이원석B</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>정경훈</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>신명철</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>최지명</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>정경배</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>윤정빈</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>진갑용</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>최충연</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>이동수S</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>강동우</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -61397,9 +61593,15 @@
       <c r="J231" s="3"/>
     </row>
     <row r="232" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A232" s="9"/>
-      <c r="B232" s="8"/>
-      <c r="C232" s="8"/>
+      <c r="A232" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B232" s="9" t="s">
+        <v>753</v>
+      </c>
+      <c r="C232" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D232" s="8"/>
       <c r="E232" s="3"/>
       <c r="F232" s="3"/>
@@ -61409,9 +61611,15 @@
       <c r="J232" s="3"/>
     </row>
     <row r="233" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A233" s="8"/>
-      <c r="B233" s="8"/>
-      <c r="C233" s="8"/>
+      <c r="A233" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B233" s="9" t="s">
+        <v>745</v>
+      </c>
+      <c r="C233" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D233" s="8"/>
       <c r="E233" s="3"/>
       <c r="F233" s="3"/>
@@ -61421,9 +61629,15 @@
       <c r="J233" s="3"/>
     </row>
     <row r="234" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A234" s="8"/>
-      <c r="B234" s="8"/>
-      <c r="C234" s="8"/>
+      <c r="A234" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B234" s="9" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C234" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D234" s="8"/>
       <c r="E234" s="3"/>
       <c r="F234" s="3"/>
@@ -61433,9 +61647,15 @@
       <c r="J234" s="3"/>
     </row>
     <row r="235" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A235" s="8"/>
-      <c r="B235" s="8"/>
-      <c r="C235" s="8"/>
+      <c r="A235" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B235" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="C235" s="9" t="s">
+        <v>1027</v>
+      </c>
       <c r="D235" s="8"/>
       <c r="E235" s="3"/>
       <c r="F235" s="3"/>
@@ -61445,9 +61665,15 @@
       <c r="J235" s="3"/>
     </row>
     <row r="236" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A236" s="8"/>
-      <c r="B236" s="8"/>
-      <c r="C236" s="8"/>
+      <c r="A236" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B236" s="9" t="s">
+        <v>751</v>
+      </c>
+      <c r="C236" s="9" t="s">
+        <v>1032</v>
+      </c>
       <c r="D236" s="8"/>
       <c r="E236" s="3"/>
       <c r="F236" s="3"/>
@@ -61457,9 +61683,15 @@
       <c r="J236" s="3"/>
     </row>
     <row r="237" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A237" s="8"/>
-      <c r="B237" s="8"/>
-      <c r="C237" s="8"/>
+      <c r="A237" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B237" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="C237" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D237" s="8"/>
       <c r="E237" s="3"/>
       <c r="F237" s="3"/>
@@ -61469,9 +61701,15 @@
       <c r="J237" s="3"/>
     </row>
     <row r="238" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A238" s="8"/>
-      <c r="B238" s="8"/>
-      <c r="C238" s="8"/>
+      <c r="A238" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B238" s="9" t="s">
+        <v>692</v>
+      </c>
+      <c r="C238" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D238" s="8"/>
       <c r="E238" s="3"/>
       <c r="F238" s="3"/>
@@ -61481,9 +61719,15 @@
       <c r="J238" s="3"/>
     </row>
     <row r="239" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A239" s="8"/>
-      <c r="B239" s="8"/>
-      <c r="C239" s="8"/>
+      <c r="A239" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B239" s="9" t="s">
+        <v>749</v>
+      </c>
+      <c r="C239" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D239" s="8"/>
       <c r="E239" s="3"/>
       <c r="F239" s="3"/>
@@ -61493,9 +61737,15 @@
       <c r="J239" s="3"/>
     </row>
     <row r="240" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A240" s="8"/>
-      <c r="B240" s="8"/>
-      <c r="C240" s="8"/>
+      <c r="A240" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B240" s="9" t="s">
+        <v>749</v>
+      </c>
+      <c r="C240" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D240" s="8"/>
       <c r="E240" s="3"/>
       <c r="F240" s="3"/>
@@ -61505,9 +61755,15 @@
       <c r="J240" s="3"/>
     </row>
     <row r="241" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A241" s="8"/>
-      <c r="B241" s="8"/>
-      <c r="C241" s="8"/>
+      <c r="A241" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B241" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="C241" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D241" s="8"/>
       <c r="E241" s="3"/>
       <c r="F241" s="3"/>
@@ -61517,9 +61773,15 @@
       <c r="J241" s="3"/>
     </row>
     <row r="242" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A242" s="8"/>
-      <c r="B242" s="8"/>
-      <c r="C242" s="8"/>
+      <c r="A242" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B242" s="10" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C242" s="10" t="s">
+        <v>1029</v>
+      </c>
       <c r="D242" s="8"/>
       <c r="E242" s="3"/>
       <c r="F242" s="3"/>
@@ -61529,9 +61791,15 @@
       <c r="J242" s="3"/>
     </row>
     <row r="243" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A243" s="8"/>
-      <c r="B243" s="8"/>
-      <c r="C243" s="8"/>
+      <c r="A243" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B243" s="10" t="s">
+        <v>1113</v>
+      </c>
+      <c r="C243" s="10" t="s">
+        <v>1032</v>
+      </c>
       <c r="D243" s="8"/>
       <c r="E243" s="3"/>
       <c r="F243" s="3"/>
@@ -61541,9 +61809,15 @@
       <c r="J243" s="3"/>
     </row>
     <row r="244" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A244" s="8"/>
-      <c r="B244" s="8"/>
-      <c r="C244" s="8"/>
+      <c r="A244" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B244" s="10" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C244" s="10" t="s">
+        <v>1043</v>
+      </c>
       <c r="D244" s="8"/>
       <c r="E244" s="3"/>
       <c r="F244" s="3"/>
@@ -61553,9 +61827,15 @@
       <c r="J244" s="3"/>
     </row>
     <row r="245" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A245" s="8"/>
-      <c r="B245" s="8"/>
-      <c r="C245" s="8"/>
+      <c r="A245" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B245" s="10" t="s">
+        <v>757</v>
+      </c>
+      <c r="C245" s="10" t="s">
+        <v>1032</v>
+      </c>
       <c r="D245" s="8"/>
       <c r="E245" s="3"/>
       <c r="F245" s="3"/>
@@ -61565,9 +61845,15 @@
       <c r="J245" s="3"/>
     </row>
     <row r="246" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A246" s="8"/>
-      <c r="B246" s="8"/>
-      <c r="C246" s="8"/>
+      <c r="A246" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B246" s="10" t="s">
+        <v>764</v>
+      </c>
+      <c r="C246" s="10" t="s">
+        <v>1039</v>
+      </c>
       <c r="D246" s="8"/>
       <c r="E246" s="3"/>
       <c r="F246" s="3"/>
@@ -61577,9 +61863,15 @@
       <c r="J246" s="3"/>
     </row>
     <row r="247" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A247" s="8"/>
-      <c r="B247" s="8"/>
-      <c r="C247" s="8"/>
+      <c r="A247" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B247" s="10" t="s">
+        <v>762</v>
+      </c>
+      <c r="C247" s="10" t="s">
+        <v>1049</v>
+      </c>
       <c r="D247" s="8"/>
       <c r="E247" s="3"/>
       <c r="F247" s="3"/>
@@ -61589,9 +61881,15 @@
       <c r="J247" s="3"/>
     </row>
     <row r="248" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A248" s="8"/>
-      <c r="B248" s="8"/>
-      <c r="C248" s="8"/>
+      <c r="A248" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B248" s="10" t="s">
+        <v>752</v>
+      </c>
+      <c r="C248" s="10" t="s">
+        <v>1040</v>
+      </c>
       <c r="D248" s="8"/>
       <c r="E248" s="3"/>
       <c r="F248" s="3"/>
@@ -61601,9 +61899,15 @@
       <c r="J248" s="3"/>
     </row>
     <row r="249" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A249" s="8"/>
-      <c r="B249" s="8"/>
-      <c r="C249" s="8"/>
+      <c r="A249" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B249" s="10" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C249" s="10" t="s">
+        <v>1031</v>
+      </c>
       <c r="D249" s="8"/>
       <c r="E249" s="3"/>
       <c r="F249" s="3"/>
@@ -61613,9 +61917,15 @@
       <c r="J249" s="3"/>
     </row>
     <row r="250" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A250" s="8"/>
-      <c r="B250" s="8"/>
-      <c r="C250" s="8"/>
+      <c r="A250" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B250" s="10" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C250" s="10" t="s">
+        <v>1031</v>
+      </c>
       <c r="D250" s="8"/>
       <c r="E250" s="3"/>
       <c r="F250" s="3"/>
@@ -61625,9 +61935,15 @@
       <c r="J250" s="3"/>
     </row>
     <row r="251" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A251" s="8"/>
-      <c r="B251" s="8"/>
-      <c r="C251" s="8"/>
+      <c r="A251" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B251" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C251" s="10" t="s">
+        <v>1043</v>
+      </c>
       <c r="D251" s="8"/>
       <c r="E251" s="3"/>
       <c r="F251" s="3"/>
@@ -61637,9 +61953,15 @@
       <c r="J251" s="3"/>
     </row>
     <row r="252" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A252" s="8"/>
-      <c r="B252" s="8"/>
-      <c r="C252" s="8"/>
+      <c r="A252" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B252" s="9" t="s">
+        <v>747</v>
+      </c>
+      <c r="C252" s="9" t="s">
+        <v>1038</v>
+      </c>
       <c r="D252" s="8"/>
       <c r="E252" s="3"/>
       <c r="F252" s="3"/>
@@ -61649,9 +61971,15 @@
       <c r="J252" s="3"/>
     </row>
     <row r="253" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A253" s="8"/>
-      <c r="B253" s="8"/>
-      <c r="C253" s="8"/>
+      <c r="A253" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B253" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="C253" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D253" s="8"/>
       <c r="E253" s="3"/>
       <c r="F253" s="3"/>
@@ -61661,9 +61989,15 @@
       <c r="J253" s="3"/>
     </row>
     <row r="254" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A254" s="8"/>
-      <c r="B254" s="8"/>
-      <c r="C254" s="8"/>
+      <c r="A254" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B254" s="9" t="s">
+        <v>754</v>
+      </c>
+      <c r="C254" s="9" t="s">
+        <v>1060</v>
+      </c>
       <c r="D254" s="8"/>
       <c r="E254" s="3"/>
       <c r="F254" s="3"/>
@@ -61673,9 +62007,15 @@
       <c r="J254" s="3"/>
     </row>
     <row r="255" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A255" s="8"/>
-      <c r="B255" s="8"/>
-      <c r="C255" s="8"/>
+      <c r="A255" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B255" s="9" t="s">
+        <v>740</v>
+      </c>
+      <c r="C255" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D255" s="8"/>
       <c r="E255" s="3"/>
       <c r="F255" s="3"/>
@@ -61685,9 +62025,15 @@
       <c r="J255" s="3"/>
     </row>
     <row r="256" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A256" s="8"/>
-      <c r="B256" s="8"/>
-      <c r="C256" s="8"/>
+      <c r="A256" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B256" s="9" t="s">
+        <v>831</v>
+      </c>
+      <c r="C256" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D256" s="8"/>
       <c r="E256" s="3"/>
       <c r="F256" s="3"/>
@@ -61697,9 +62043,15 @@
       <c r="J256" s="3"/>
     </row>
     <row r="257" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A257" s="8"/>
-      <c r="B257" s="8"/>
-      <c r="C257" s="8"/>
+      <c r="A257" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B257" s="9" t="s">
+        <v>761</v>
+      </c>
+      <c r="C257" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D257" s="8"/>
       <c r="E257" s="3"/>
       <c r="F257" s="3"/>
@@ -61709,9 +62061,15 @@
       <c r="J257" s="3"/>
     </row>
     <row r="258" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A258" s="8"/>
-      <c r="B258" s="8"/>
-      <c r="C258" s="8"/>
+      <c r="A258" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B258" s="9" t="s">
+        <v>1117</v>
+      </c>
+      <c r="C258" s="9" t="s">
+        <v>1061</v>
+      </c>
       <c r="D258" s="8"/>
       <c r="E258" s="3"/>
       <c r="F258" s="3"/>
@@ -61721,9 +62079,15 @@
       <c r="J258" s="3"/>
     </row>
     <row r="259" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A259" s="8"/>
-      <c r="B259" s="8"/>
-      <c r="C259" s="8"/>
+      <c r="A259" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B259" s="9" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C259" s="9" t="s">
+        <v>1066</v>
+      </c>
       <c r="D259" s="8"/>
       <c r="E259" s="3"/>
       <c r="F259" s="3"/>
@@ -61733,9 +62097,15 @@
       <c r="J259" s="3"/>
     </row>
     <row r="260" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A260" s="8"/>
-      <c r="B260" s="8"/>
-      <c r="C260" s="8"/>
+      <c r="A260" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B260" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C260" s="9" t="s">
+        <v>1071</v>
+      </c>
       <c r="D260" s="8"/>
       <c r="E260" s="3"/>
       <c r="F260" s="3"/>
@@ -61745,9 +62115,15 @@
       <c r="J260" s="3"/>
     </row>
     <row r="261" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A261" s="8"/>
-      <c r="B261" s="8"/>
-      <c r="C261" s="8"/>
+      <c r="A261" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B261" s="9" t="s">
+        <v>959</v>
+      </c>
+      <c r="C261" s="9" t="s">
+        <v>1048</v>
+      </c>
       <c r="D261" s="8"/>
       <c r="E261" s="3"/>
       <c r="F261" s="3"/>
@@ -61757,9 +62133,15 @@
       <c r="J261" s="3"/>
     </row>
     <row r="262" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A262" s="8"/>
-      <c r="B262" s="8"/>
-      <c r="C262" s="8"/>
+      <c r="A262" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B262" s="9" t="s">
+        <v>1120</v>
+      </c>
+      <c r="C262" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D262" s="8"/>
       <c r="E262" s="3"/>
       <c r="F262" s="3"/>
@@ -61769,9 +62151,15 @@
       <c r="J262" s="3"/>
     </row>
     <row r="263" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A263" s="8"/>
-      <c r="B263" s="8"/>
-      <c r="C263" s="8"/>
+      <c r="A263" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B263" s="9" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C263" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D263" s="8"/>
       <c r="E263" s="3"/>
       <c r="F263" s="3"/>
@@ -61781,9 +62169,15 @@
       <c r="J263" s="3"/>
     </row>
     <row r="264" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A264" s="8"/>
-      <c r="B264" s="8"/>
-      <c r="C264" s="8"/>
+      <c r="A264" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B264" s="9" t="s">
+        <v>868</v>
+      </c>
+      <c r="C264" s="9" t="s">
+        <v>1038</v>
+      </c>
       <c r="D264" s="8"/>
       <c r="E264" s="3"/>
       <c r="F264" s="3"/>
@@ -61793,9 +62187,15 @@
       <c r="J264" s="3"/>
     </row>
     <row r="265" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A265" s="8"/>
-      <c r="B265" s="8"/>
-      <c r="C265" s="8"/>
+      <c r="A265" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B265" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C265" s="9" t="s">
+        <v>1040</v>
+      </c>
       <c r="D265" s="8"/>
       <c r="E265" s="3"/>
       <c r="F265" s="3"/>
@@ -61805,9 +62205,15 @@
       <c r="J265" s="3"/>
     </row>
     <row r="266" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A266" s="8"/>
-      <c r="B266" s="8"/>
-      <c r="C266" s="8"/>
+      <c r="A266" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B266" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C266" s="9" t="s">
+        <v>1051</v>
+      </c>
       <c r="D266" s="8"/>
       <c r="E266" s="3"/>
       <c r="F266" s="3"/>
@@ -61817,9 +62223,15 @@
       <c r="J266" s="3"/>
     </row>
     <row r="267" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A267" s="8"/>
-      <c r="B267" s="8"/>
-      <c r="C267" s="8"/>
+      <c r="A267" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B267" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="C267" s="9" t="s">
+        <v>1076</v>
+      </c>
       <c r="D267" s="8"/>
       <c r="E267" s="3"/>
       <c r="F267" s="3"/>
@@ -61829,9 +62241,15 @@
       <c r="J267" s="3"/>
     </row>
     <row r="268" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A268" s="8"/>
-      <c r="B268" s="8"/>
-      <c r="C268" s="8"/>
+      <c r="A268" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B268" s="9" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C268" s="10" t="s">
+        <v>1041</v>
+      </c>
       <c r="D268" s="8"/>
       <c r="E268" s="3"/>
       <c r="F268" s="3"/>
@@ -61841,9 +62259,15 @@
       <c r="J268" s="3"/>
     </row>
     <row r="269" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A269" s="8"/>
-      <c r="B269" s="8"/>
-      <c r="C269" s="8"/>
+      <c r="A269" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B269" s="9" t="s">
+        <v>1122</v>
+      </c>
+      <c r="C269" s="9" t="s">
+        <v>1041</v>
+      </c>
       <c r="D269" s="8"/>
       <c r="E269" s="3"/>
       <c r="F269" s="3"/>
@@ -61853,9 +62277,15 @@
       <c r="J269" s="3"/>
     </row>
     <row r="270" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A270" s="8"/>
-      <c r="B270" s="8"/>
-      <c r="C270" s="8"/>
+      <c r="A270" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B270" s="9" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C270" s="9" t="s">
+        <v>1041</v>
+      </c>
       <c r="D270" s="8"/>
       <c r="E270" s="3"/>
       <c r="F270" s="3"/>
@@ -61865,9 +62295,15 @@
       <c r="J270" s="3"/>
     </row>
     <row r="271" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A271" s="8"/>
-      <c r="B271" s="8"/>
-      <c r="C271" s="8"/>
+      <c r="A271" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B271" s="9" t="s">
+        <v>1112</v>
+      </c>
+      <c r="C271" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D271" s="8"/>
       <c r="E271" s="3"/>
       <c r="F271" s="3"/>
@@ -61877,9 +62313,15 @@
       <c r="J271" s="3"/>
     </row>
     <row r="272" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A272" s="8"/>
-      <c r="B272" s="8"/>
-      <c r="C272" s="8"/>
+      <c r="A272" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B272" s="9" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C272" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D272" s="8"/>
       <c r="E272" s="3"/>
       <c r="F272" s="3"/>
@@ -61889,9 +62331,15 @@
       <c r="J272" s="3"/>
     </row>
     <row r="273" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A273" s="8"/>
-      <c r="B273" s="8"/>
-      <c r="C273" s="8"/>
+      <c r="A273" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B273" s="9" t="s">
+        <v>764</v>
+      </c>
+      <c r="C273" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D273" s="8"/>
       <c r="E273" s="3"/>
       <c r="F273" s="3"/>
@@ -61901,9 +62349,15 @@
       <c r="J273" s="3"/>
     </row>
     <row r="274" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A274" s="8"/>
-      <c r="B274" s="8"/>
-      <c r="C274" s="8"/>
+      <c r="A274" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B274" s="9" t="s">
+        <v>746</v>
+      </c>
+      <c r="C274" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D274" s="8"/>
       <c r="E274" s="3"/>
       <c r="F274" s="3"/>
@@ -61913,9 +62367,15 @@
       <c r="J274" s="3"/>
     </row>
     <row r="275" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A275" s="8"/>
-      <c r="B275" s="8"/>
-      <c r="C275" s="8"/>
+      <c r="A275" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B275" s="9" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C275" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D275" s="8"/>
       <c r="E275" s="3"/>
       <c r="F275" s="3"/>
@@ -61925,9 +62385,15 @@
       <c r="J275" s="3"/>
     </row>
     <row r="276" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A276" s="8"/>
-      <c r="B276" s="8"/>
-      <c r="C276" s="8"/>
+      <c r="A276" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B276" s="9" t="s">
+        <v>678</v>
+      </c>
+      <c r="C276" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D276" s="8"/>
       <c r="E276" s="3"/>
       <c r="F276" s="3"/>
@@ -61937,9 +62403,15 @@
       <c r="J276" s="3"/>
     </row>
     <row r="277" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A277" s="8"/>
-      <c r="B277" s="8"/>
-      <c r="C277" s="8"/>
+      <c r="A277" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B277" s="9" t="s">
+        <v>742</v>
+      </c>
+      <c r="C277" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D277" s="8"/>
       <c r="E277" s="3"/>
       <c r="F277" s="3"/>
@@ -61949,9 +62421,15 @@
       <c r="J277" s="3"/>
     </row>
     <row r="278" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A278" s="8"/>
-      <c r="B278" s="8"/>
-      <c r="C278" s="8"/>
+      <c r="A278" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B278" s="9" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C278" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D278" s="8"/>
       <c r="E278" s="3"/>
       <c r="F278" s="3"/>
@@ -61961,9 +62439,15 @@
       <c r="J278" s="3"/>
     </row>
     <row r="279" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A279" s="8"/>
-      <c r="B279" s="8"/>
-      <c r="C279" s="8"/>
+      <c r="A279" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B279" s="9" t="s">
+        <v>1126</v>
+      </c>
+      <c r="C279" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D279" s="8"/>
       <c r="E279" s="3"/>
       <c r="F279" s="3"/>
@@ -61973,9 +62457,15 @@
       <c r="J279" s="3"/>
     </row>
     <row r="280" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A280" s="8"/>
-      <c r="B280" s="8"/>
-      <c r="C280" s="8"/>
+      <c r="A280" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B280" s="10" t="s">
+        <v>742</v>
+      </c>
+      <c r="C280" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D280" s="8"/>
       <c r="E280" s="3"/>
       <c r="F280" s="3"/>
@@ -61985,9 +62475,15 @@
       <c r="J280" s="3"/>
     </row>
     <row r="281" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A281" s="8"/>
-      <c r="B281" s="8"/>
-      <c r="C281" s="8"/>
+      <c r="A281" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B281" s="9" t="s">
+        <v>754</v>
+      </c>
+      <c r="C281" s="9" t="s">
+        <v>1032</v>
+      </c>
       <c r="D281" s="8"/>
       <c r="E281" s="3"/>
       <c r="F281" s="3"/>
@@ -61997,9 +62493,15 @@
       <c r="J281" s="3"/>
     </row>
     <row r="282" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A282" s="8"/>
-      <c r="B282" s="8"/>
-      <c r="C282" s="8"/>
+      <c r="A282" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B282" s="9" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C282" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D282" s="8"/>
       <c r="E282" s="3"/>
       <c r="F282" s="3"/>
@@ -62009,9 +62511,15 @@
       <c r="J282" s="3"/>
     </row>
     <row r="283" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A283" s="8"/>
-      <c r="B283" s="8"/>
-      <c r="C283" s="8"/>
+      <c r="A283" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B283" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="C283" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D283" s="8"/>
       <c r="E283" s="3"/>
       <c r="F283" s="3"/>
@@ -62021,9 +62529,15 @@
       <c r="J283" s="3"/>
     </row>
     <row r="284" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A284" s="8"/>
-      <c r="B284" s="8"/>
-      <c r="C284" s="8"/>
+      <c r="A284" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B284" s="9" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C284" s="9" t="s">
+        <v>1062</v>
+      </c>
       <c r="D284" s="8"/>
       <c r="E284" s="3"/>
       <c r="F284" s="3"/>
@@ -62033,9 +62547,15 @@
       <c r="J284" s="3"/>
     </row>
     <row r="285" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A285" s="8"/>
-      <c r="B285" s="8"/>
-      <c r="C285" s="8"/>
+      <c r="A285" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B285" s="9" t="s">
+        <v>1129</v>
+      </c>
+      <c r="C285" s="9" t="s">
+        <v>1062</v>
+      </c>
       <c r="D285" s="8"/>
       <c r="E285" s="3"/>
       <c r="F285" s="3"/>
@@ -62045,9 +62565,15 @@
       <c r="J285" s="3"/>
     </row>
     <row r="286" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A286" s="8"/>
-      <c r="B286" s="8"/>
-      <c r="C286" s="8"/>
+      <c r="A286" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B286" s="9" t="s">
+        <v>772</v>
+      </c>
+      <c r="C286" s="9" t="s">
+        <v>1056</v>
+      </c>
       <c r="D286" s="8"/>
       <c r="E286" s="3"/>
       <c r="F286" s="3"/>
@@ -62057,9 +62583,15 @@
       <c r="J286" s="3"/>
     </row>
     <row r="287" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A287" s="8"/>
-      <c r="B287" s="8"/>
-      <c r="C287" s="8"/>
+      <c r="A287" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B287" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C287" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D287" s="8"/>
       <c r="E287" s="3"/>
       <c r="F287" s="3"/>
@@ -62069,9 +62601,15 @@
       <c r="J287" s="3"/>
     </row>
     <row r="288" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A288" s="8"/>
-      <c r="B288" s="8"/>
-      <c r="C288" s="8"/>
+      <c r="A288" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B288" s="9" t="s">
+        <v>759</v>
+      </c>
+      <c r="C288" s="9" t="s">
+        <v>1027</v>
+      </c>
       <c r="D288" s="8"/>
       <c r="E288" s="3"/>
       <c r="F288" s="3"/>
@@ -62081,9 +62619,15 @@
       <c r="J288" s="3"/>
     </row>
     <row r="289" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A289" s="8"/>
-      <c r="B289" s="8"/>
-      <c r="C289" s="8"/>
+      <c r="A289" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B289" s="10" t="s">
+        <v>771</v>
+      </c>
+      <c r="C289" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D289" s="8"/>
       <c r="E289" s="3"/>
       <c r="F289" s="3"/>
@@ -62093,9 +62637,15 @@
       <c r="J289" s="3"/>
     </row>
     <row r="290" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A290" s="8"/>
-      <c r="B290" s="8"/>
-      <c r="C290" s="8"/>
+      <c r="A290" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B290" s="9" t="s">
+        <v>1130</v>
+      </c>
+      <c r="C290" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D290" s="8"/>
       <c r="E290" s="3"/>
       <c r="F290" s="3"/>
@@ -62105,9 +62655,15 @@
       <c r="J290" s="3"/>
     </row>
     <row r="291" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A291" s="8"/>
-      <c r="B291" s="8"/>
-      <c r="C291" s="8"/>
+      <c r="A291" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B291" s="9" t="s">
+        <v>745</v>
+      </c>
+      <c r="C291" s="9" t="s">
+        <v>1061</v>
+      </c>
       <c r="D291" s="8"/>
       <c r="E291" s="3"/>
       <c r="F291" s="3"/>
@@ -62117,9 +62673,15 @@
       <c r="J291" s="3"/>
     </row>
     <row r="292" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A292" s="8"/>
-      <c r="B292" s="8"/>
-      <c r="C292" s="8"/>
+      <c r="A292" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B292" s="9" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C292" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D292" s="8"/>
       <c r="E292" s="3"/>
       <c r="F292" s="3"/>
@@ -62129,9 +62691,15 @@
       <c r="J292" s="3"/>
     </row>
     <row r="293" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A293" s="8"/>
-      <c r="B293" s="8"/>
-      <c r="C293" s="8"/>
+      <c r="A293" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B293" s="9" t="s">
+        <v>752</v>
+      </c>
+      <c r="C293" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D293" s="8"/>
       <c r="E293" s="3"/>
       <c r="F293" s="3"/>
@@ -62141,9 +62709,15 @@
       <c r="J293" s="3"/>
     </row>
     <row r="294" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A294" s="8"/>
-      <c r="B294" s="8"/>
-      <c r="C294" s="8"/>
+      <c r="A294" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B294" s="9" t="s">
+        <v>745</v>
+      </c>
+      <c r="C294" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D294" s="8"/>
       <c r="E294" s="3"/>
       <c r="F294" s="3"/>
@@ -62153,9 +62727,15 @@
       <c r="J294" s="3"/>
     </row>
     <row r="295" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A295" s="8"/>
-      <c r="B295" s="8"/>
-      <c r="C295" s="8"/>
+      <c r="A295" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B295" s="9" t="s">
+        <v>746</v>
+      </c>
+      <c r="C295" s="9" t="s">
+        <v>1056</v>
+      </c>
       <c r="D295" s="8"/>
       <c r="E295" s="3"/>
       <c r="F295" s="3"/>
@@ -62165,9 +62745,15 @@
       <c r="J295" s="3"/>
     </row>
     <row r="296" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A296" s="8"/>
-      <c r="B296" s="8"/>
-      <c r="C296" s="8"/>
+      <c r="A296" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B296" s="9" t="s">
+        <v>662</v>
+      </c>
+      <c r="C296" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D296" s="8"/>
       <c r="E296" s="3"/>
       <c r="F296" s="3"/>
@@ -62177,9 +62763,15 @@
       <c r="J296" s="3"/>
     </row>
     <row r="297" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A297" s="8"/>
-      <c r="B297" s="8"/>
-      <c r="C297" s="8"/>
+      <c r="A297" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B297" s="9" t="s">
+        <v>1131</v>
+      </c>
+      <c r="C297" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D297" s="8"/>
       <c r="E297" s="3"/>
       <c r="F297" s="3"/>
@@ -62189,9 +62781,15 @@
       <c r="J297" s="3"/>
     </row>
     <row r="298" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A298" s="8"/>
-      <c r="B298" s="8"/>
-      <c r="C298" s="8"/>
+      <c r="A298" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B298" s="9" t="s">
+        <v>744</v>
+      </c>
+      <c r="C298" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D298" s="8"/>
       <c r="E298" s="3"/>
       <c r="F298" s="3"/>
@@ -62201,9 +62799,15 @@
       <c r="J298" s="3"/>
     </row>
     <row r="299" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A299" s="8"/>
-      <c r="B299" s="8"/>
-      <c r="C299" s="8"/>
+      <c r="A299" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B299" s="9" t="s">
+        <v>983</v>
+      </c>
+      <c r="C299" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D299" s="8"/>
       <c r="E299" s="3"/>
       <c r="F299" s="3"/>
@@ -62213,9 +62817,15 @@
       <c r="J299" s="3"/>
     </row>
     <row r="300" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A300" s="8"/>
-      <c r="B300" s="8"/>
-      <c r="C300" s="8"/>
+      <c r="A300" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B300" s="9" t="s">
+        <v>771</v>
+      </c>
+      <c r="C300" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D300" s="8"/>
       <c r="E300" s="3"/>
       <c r="F300" s="3"/>
@@ -62225,9 +62835,15 @@
       <c r="J300" s="3"/>
     </row>
     <row r="301" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A301" s="8"/>
-      <c r="B301" s="8"/>
-      <c r="C301" s="8"/>
+      <c r="A301" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B301" s="9" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C301" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D301" s="8"/>
       <c r="E301" s="3"/>
       <c r="F301" s="3"/>
@@ -62237,9 +62853,15 @@
       <c r="J301" s="3"/>
     </row>
     <row r="302" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A302" s="8"/>
-      <c r="B302" s="8"/>
-      <c r="C302" s="8"/>
+      <c r="A302" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B302" s="9" t="s">
+        <v>742</v>
+      </c>
+      <c r="C302" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D302" s="8"/>
       <c r="E302" s="3"/>
       <c r="F302" s="3"/>
@@ -62249,9 +62871,15 @@
       <c r="J302" s="3"/>
     </row>
     <row r="303" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A303" s="8"/>
-      <c r="B303" s="8"/>
-      <c r="C303" s="8"/>
+      <c r="A303" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B303" s="9" t="s">
+        <v>1132</v>
+      </c>
+      <c r="C303" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D303" s="8"/>
       <c r="E303" s="3"/>
       <c r="F303" s="3"/>
@@ -62261,9 +62889,15 @@
       <c r="J303" s="3"/>
     </row>
     <row r="304" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A304" s="8"/>
-      <c r="B304" s="8"/>
-      <c r="C304" s="8"/>
+      <c r="A304" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B304" s="9" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C304" s="9" t="s">
+        <v>1032</v>
+      </c>
       <c r="D304" s="8"/>
       <c r="E304" s="3"/>
       <c r="F304" s="3"/>
@@ -62273,9 +62907,15 @@
       <c r="J304" s="3"/>
     </row>
     <row r="305" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A305" s="8"/>
-      <c r="B305" s="8"/>
-      <c r="C305" s="8"/>
+      <c r="A305" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B305" s="9" t="s">
+        <v>755</v>
+      </c>
+      <c r="C305" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D305" s="8"/>
       <c r="E305" s="3"/>
       <c r="F305" s="3"/>
@@ -62285,9 +62925,15 @@
       <c r="J305" s="3"/>
     </row>
     <row r="306" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A306" s="8"/>
-      <c r="B306" s="8"/>
-      <c r="C306" s="8"/>
+      <c r="A306" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B306" s="9" t="s">
+        <v>747</v>
+      </c>
+      <c r="C306" s="9" t="s">
+        <v>1032</v>
+      </c>
       <c r="D306" s="8"/>
       <c r="E306" s="3"/>
       <c r="F306" s="3"/>
@@ -62297,9 +62943,15 @@
       <c r="J306" s="3"/>
     </row>
     <row r="307" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A307" s="8"/>
-      <c r="B307" s="8"/>
-      <c r="C307" s="8"/>
+      <c r="A307" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B307" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C307" s="9" t="s">
+        <v>1060</v>
+      </c>
       <c r="D307" s="8"/>
       <c r="E307" s="3"/>
       <c r="F307" s="3"/>
@@ -62309,9 +62961,15 @@
       <c r="J307" s="3"/>
     </row>
     <row r="308" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A308" s="8"/>
-      <c r="B308" s="8"/>
-      <c r="C308" s="8"/>
+      <c r="A308" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B308" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C308" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D308" s="8"/>
       <c r="E308" s="3"/>
       <c r="F308" s="3"/>
@@ -62321,9 +62979,15 @@
       <c r="J308" s="3"/>
     </row>
     <row r="309" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A309" s="8"/>
-      <c r="B309" s="8"/>
-      <c r="C309" s="8"/>
+      <c r="A309" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B309" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C309" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D309" s="8"/>
       <c r="E309" s="3"/>
       <c r="F309" s="3"/>
@@ -62333,9 +62997,15 @@
       <c r="J309" s="3"/>
     </row>
     <row r="310" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A310" s="8"/>
-      <c r="B310" s="8"/>
-      <c r="C310" s="8"/>
+      <c r="A310" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B310" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="C310" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D310" s="8"/>
       <c r="E310" s="3"/>
       <c r="F310" s="3"/>
@@ -62345,9 +63015,15 @@
       <c r="J310" s="3"/>
     </row>
     <row r="311" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A311" s="8"/>
-      <c r="B311" s="8"/>
-      <c r="C311" s="8"/>
+      <c r="A311" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B311" s="9" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C311" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D311" s="8"/>
       <c r="E311" s="3"/>
       <c r="F311" s="3"/>
@@ -62357,9 +63033,15 @@
       <c r="J311" s="3"/>
     </row>
     <row r="312" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A312" s="8"/>
-      <c r="B312" s="8"/>
-      <c r="C312" s="8"/>
+      <c r="A312" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B312" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C312" s="9" t="s">
+        <v>1070</v>
+      </c>
       <c r="D312" s="8"/>
       <c r="E312" s="3"/>
       <c r="F312" s="3"/>
@@ -62369,9 +63051,15 @@
       <c r="J312" s="3"/>
     </row>
     <row r="313" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A313" s="8"/>
-      <c r="B313" s="8"/>
-      <c r="C313" s="8"/>
+      <c r="A313" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B313" s="9" t="s">
+        <v>831</v>
+      </c>
+      <c r="C313" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D313" s="8"/>
       <c r="E313" s="3"/>
       <c r="F313" s="3"/>
@@ -62381,9 +63069,15 @@
       <c r="J313" s="3"/>
     </row>
     <row r="314" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A314" s="8"/>
-      <c r="B314" s="8"/>
-      <c r="C314" s="8"/>
+      <c r="A314" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B314" s="9" t="s">
+        <v>1133</v>
+      </c>
+      <c r="C314" s="9" t="s">
+        <v>1027</v>
+      </c>
       <c r="D314" s="8"/>
       <c r="E314" s="3"/>
       <c r="F314" s="3"/>
@@ -62393,9 +63087,15 @@
       <c r="J314" s="3"/>
     </row>
     <row r="315" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A315" s="8"/>
-      <c r="B315" s="8"/>
-      <c r="C315" s="8"/>
+      <c r="A315" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B315" s="9" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C315" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D315" s="8"/>
       <c r="E315" s="3"/>
       <c r="F315" s="3"/>
@@ -62405,9 +63105,15 @@
       <c r="J315" s="3"/>
     </row>
     <row r="316" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A316" s="8"/>
-      <c r="B316" s="8"/>
-      <c r="C316" s="8"/>
+      <c r="A316" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B316" s="9" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C316" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D316" s="8"/>
       <c r="E316" s="3"/>
       <c r="F316" s="3"/>
@@ -62417,9 +63123,15 @@
       <c r="J316" s="3"/>
     </row>
     <row r="317" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A317" s="8"/>
-      <c r="B317" s="8"/>
-      <c r="C317" s="8"/>
+      <c r="A317" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B317" s="9" t="s">
+        <v>1136</v>
+      </c>
+      <c r="C317" s="10" t="s">
+        <v>1039</v>
+      </c>
       <c r="D317" s="8"/>
       <c r="E317" s="3"/>
       <c r="F317" s="3"/>
@@ -62429,9 +63141,15 @@
       <c r="J317" s="3"/>
     </row>
     <row r="318" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A318" s="8"/>
-      <c r="B318" s="8"/>
-      <c r="C318" s="8"/>
+      <c r="A318" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B318" s="9" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C318" s="10" t="s">
+        <v>1049</v>
+      </c>
       <c r="D318" s="8"/>
       <c r="E318" s="3"/>
       <c r="F318" s="3"/>
@@ -62441,9 +63159,15 @@
       <c r="J318" s="3"/>
     </row>
     <row r="319" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A319" s="8"/>
-      <c r="B319" s="8"/>
-      <c r="C319" s="8"/>
+      <c r="A319" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B319" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="C319" s="10" t="s">
+        <v>1075</v>
+      </c>
       <c r="D319" s="8"/>
       <c r="E319" s="3"/>
       <c r="F319" s="3"/>
@@ -62453,9 +63177,15 @@
       <c r="J319" s="3"/>
     </row>
     <row r="320" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A320" s="8"/>
-      <c r="B320" s="8"/>
-      <c r="C320" s="8"/>
+      <c r="A320" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B320" s="9" t="s">
+        <v>745</v>
+      </c>
+      <c r="C320" s="10" t="s">
+        <v>1040</v>
+      </c>
       <c r="D320" s="8"/>
       <c r="E320" s="3"/>
       <c r="F320" s="3"/>
@@ -62465,9 +63195,15 @@
       <c r="J320" s="3"/>
     </row>
     <row r="321" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A321" s="8"/>
-      <c r="B321" s="8"/>
-      <c r="C321" s="8"/>
+      <c r="A321" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B321" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C321" s="10" t="s">
+        <v>1061</v>
+      </c>
       <c r="D321" s="8"/>
       <c r="E321" s="3"/>
       <c r="F321" s="3"/>
@@ -62477,9 +63213,15 @@
       <c r="J321" s="3"/>
     </row>
     <row r="322" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A322" s="8"/>
-      <c r="B322" s="8"/>
-      <c r="C322" s="8"/>
+      <c r="A322" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B322" s="9" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C322" s="10" t="s">
+        <v>1076</v>
+      </c>
       <c r="D322" s="8"/>
       <c r="E322" s="3"/>
       <c r="F322" s="3"/>
@@ -62489,9 +63231,15 @@
       <c r="J322" s="3"/>
     </row>
     <row r="323" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A323" s="8"/>
-      <c r="B323" s="8"/>
-      <c r="C323" s="8"/>
+      <c r="A323" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B323" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="C323" s="10" t="s">
+        <v>1041</v>
+      </c>
       <c r="D323" s="8"/>
       <c r="E323" s="3"/>
       <c r="F323" s="3"/>
@@ -62501,9 +63249,15 @@
       <c r="J323" s="3"/>
     </row>
     <row r="324" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A324" s="8"/>
-      <c r="B324" s="8"/>
-      <c r="C324" s="8"/>
+      <c r="A324" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B324" s="9" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C324" s="10" t="s">
+        <v>1077</v>
+      </c>
       <c r="D324" s="8"/>
       <c r="E324" s="3"/>
       <c r="F324" s="3"/>
@@ -62513,9 +63267,15 @@
       <c r="J324" s="3"/>
     </row>
     <row r="325" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A325" s="8"/>
-      <c r="B325" s="8"/>
-      <c r="C325" s="8"/>
+      <c r="A325" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B325" s="9" t="s">
+        <v>764</v>
+      </c>
+      <c r="C325" s="10" t="s">
+        <v>1069</v>
+      </c>
       <c r="D325" s="8"/>
       <c r="E325" s="3"/>
       <c r="F325" s="3"/>
@@ -62525,9 +63285,15 @@
       <c r="J325" s="3"/>
     </row>
     <row r="326" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A326" s="8"/>
-      <c r="B326" s="8"/>
-      <c r="C326" s="8"/>
+      <c r="A326" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B326" s="9" t="s">
+        <v>766</v>
+      </c>
+      <c r="C326" s="10" t="s">
+        <v>1046</v>
+      </c>
       <c r="D326" s="8"/>
       <c r="E326" s="3"/>
       <c r="F326" s="3"/>
@@ -62537,9 +63303,15 @@
       <c r="J326" s="3"/>
     </row>
     <row r="327" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A327" s="8"/>
-      <c r="B327" s="8"/>
-      <c r="C327" s="8"/>
+      <c r="A327" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B327" s="9" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C327" s="10" t="s">
+        <v>1046</v>
+      </c>
       <c r="D327" s="8"/>
       <c r="E327" s="3"/>
       <c r="F327" s="3"/>
@@ -62549,9 +63321,15 @@
       <c r="J327" s="3"/>
     </row>
     <row r="328" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A328" s="8"/>
-      <c r="B328" s="8"/>
-      <c r="C328" s="8"/>
+      <c r="A328" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B328" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C328" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D328" s="8"/>
       <c r="E328" s="3"/>
       <c r="F328" s="3"/>
@@ -62561,9 +63339,15 @@
       <c r="J328" s="3"/>
     </row>
     <row r="329" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A329" s="8"/>
-      <c r="B329" s="8"/>
-      <c r="C329" s="8"/>
+      <c r="A329" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B329" s="9" t="s">
+        <v>1115</v>
+      </c>
+      <c r="C329" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D329" s="8"/>
       <c r="E329" s="3"/>
       <c r="F329" s="3"/>
@@ -62573,9 +63357,15 @@
       <c r="J329" s="3"/>
     </row>
     <row r="330" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A330" s="8"/>
-      <c r="B330" s="8"/>
-      <c r="C330" s="8"/>
+      <c r="A330" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B330" s="9" t="s">
+        <v>746</v>
+      </c>
+      <c r="C330" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D330" s="8"/>
       <c r="E330" s="3"/>
       <c r="F330" s="3"/>
@@ -62585,9 +63375,15 @@
       <c r="J330" s="3"/>
     </row>
     <row r="331" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A331" s="8"/>
-      <c r="B331" s="8"/>
-      <c r="C331" s="8"/>
+      <c r="A331" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B331" s="9" t="s">
+        <v>762</v>
+      </c>
+      <c r="C331" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D331" s="8"/>
       <c r="E331" s="3"/>
       <c r="F331" s="3"/>
@@ -62597,9 +63393,15 @@
       <c r="J331" s="3"/>
     </row>
     <row r="332" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A332" s="8"/>
-      <c r="B332" s="8"/>
-      <c r="C332" s="8"/>
+      <c r="A332" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B332" s="9" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C332" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D332" s="8"/>
       <c r="E332" s="3"/>
       <c r="F332" s="3"/>
@@ -62609,9 +63411,15 @@
       <c r="J332" s="3"/>
     </row>
     <row r="333" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A333" s="8"/>
-      <c r="B333" s="8"/>
-      <c r="C333" s="8"/>
+      <c r="A333" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B333" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C333" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D333" s="8"/>
       <c r="E333" s="3"/>
       <c r="F333" s="3"/>
@@ -62621,9 +63429,15 @@
       <c r="J333" s="3"/>
     </row>
     <row r="334" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A334" s="8"/>
-      <c r="B334" s="8"/>
-      <c r="C334" s="8"/>
+      <c r="A334" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B334" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C334" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D334" s="8"/>
       <c r="E334" s="3"/>
       <c r="F334" s="3"/>
@@ -62633,9 +63447,15 @@
       <c r="J334" s="3"/>
     </row>
     <row r="335" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A335" s="8"/>
-      <c r="B335" s="8"/>
-      <c r="C335" s="8"/>
+      <c r="A335" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B335" s="9" t="s">
+        <v>748</v>
+      </c>
+      <c r="C335" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D335" s="8"/>
       <c r="E335" s="3"/>
       <c r="F335" s="3"/>
@@ -62645,9 +63465,15 @@
       <c r="J335" s="3"/>
     </row>
     <row r="336" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A336" s="8"/>
-      <c r="B336" s="8"/>
-      <c r="C336" s="8"/>
+      <c r="A336" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B336" s="9" t="s">
+        <v>933</v>
+      </c>
+      <c r="C336" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D336" s="8"/>
       <c r="E336" s="3"/>
       <c r="F336" s="3"/>
@@ -62657,9 +63483,15 @@
       <c r="J336" s="3"/>
     </row>
     <row r="337" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A337" s="8"/>
-      <c r="B337" s="8"/>
-      <c r="C337" s="8"/>
+      <c r="A337" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B337" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C337" s="9" t="s">
+        <v>1060</v>
+      </c>
       <c r="D337" s="8"/>
       <c r="E337" s="3"/>
       <c r="F337" s="3"/>
@@ -62669,9 +63501,15 @@
       <c r="J337" s="3"/>
     </row>
     <row r="338" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A338" s="8"/>
-      <c r="B338" s="8"/>
-      <c r="C338" s="8"/>
+      <c r="A338" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B338" s="9" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C338" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D338" s="8"/>
       <c r="E338" s="3"/>
       <c r="F338" s="3"/>
@@ -62681,9 +63519,15 @@
       <c r="J338" s="3"/>
     </row>
     <row r="339" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A339" s="8"/>
-      <c r="B339" s="8"/>
-      <c r="C339" s="8"/>
+      <c r="A339" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B339" s="9" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C339" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D339" s="8"/>
       <c r="E339" s="3"/>
       <c r="F339" s="3"/>
@@ -62693,9 +63537,15 @@
       <c r="J339" s="3"/>
     </row>
     <row r="340" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A340" s="8"/>
-      <c r="B340" s="8"/>
-      <c r="C340" s="8"/>
+      <c r="A340" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B340" s="9" t="s">
+        <v>1124</v>
+      </c>
+      <c r="C340" s="9" t="s">
+        <v>1061</v>
+      </c>
       <c r="D340" s="8"/>
       <c r="E340" s="3"/>
       <c r="F340" s="3"/>
@@ -62705,9 +63555,15 @@
       <c r="J340" s="3"/>
     </row>
     <row r="341" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A341" s="8"/>
-      <c r="B341" s="8"/>
-      <c r="C341" s="8"/>
+      <c r="A341" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B341" s="9" t="s">
+        <v>933</v>
+      </c>
+      <c r="C341" s="9" t="s">
+        <v>1061</v>
+      </c>
       <c r="D341" s="8"/>
       <c r="E341" s="3"/>
       <c r="F341" s="3"/>
@@ -62717,9 +63573,15 @@
       <c r="J341" s="3"/>
     </row>
     <row r="342" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A342" s="8"/>
-      <c r="B342" s="8"/>
-      <c r="C342" s="8"/>
+      <c r="A342" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B342" s="9" t="s">
+        <v>1083</v>
+      </c>
+      <c r="C342" s="9" t="s">
+        <v>1071</v>
+      </c>
       <c r="D342" s="8"/>
       <c r="E342" s="3"/>
       <c r="F342" s="3"/>
@@ -62729,9 +63591,15 @@
       <c r="J342" s="3"/>
     </row>
     <row r="343" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A343" s="8"/>
-      <c r="B343" s="8"/>
-      <c r="C343" s="8"/>
+      <c r="A343" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B343" s="9" t="s">
+        <v>772</v>
+      </c>
+      <c r="C343" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D343" s="8"/>
       <c r="E343" s="3"/>
       <c r="F343" s="3"/>
@@ -62741,9 +63609,15 @@
       <c r="J343" s="3"/>
     </row>
     <row r="344" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A344" s="8"/>
-      <c r="B344" s="8"/>
-      <c r="C344" s="8"/>
+      <c r="A344" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B344" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="C344" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D344" s="8"/>
       <c r="E344" s="3"/>
       <c r="F344" s="3"/>
@@ -62753,9 +63627,15 @@
       <c r="J344" s="3"/>
     </row>
     <row r="345" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A345" s="8"/>
-      <c r="B345" s="8"/>
-      <c r="C345" s="8"/>
+      <c r="A345" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B345" s="9" t="s">
+        <v>772</v>
+      </c>
+      <c r="C345" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D345" s="8"/>
       <c r="E345" s="3"/>
       <c r="F345" s="3"/>
@@ -62765,9 +63645,15 @@
       <c r="J345" s="3"/>
     </row>
     <row r="346" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A346" s="8"/>
-      <c r="B346" s="8"/>
-      <c r="C346" s="8"/>
+      <c r="A346" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B346" s="9" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C346" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D346" s="8"/>
       <c r="E346" s="3"/>
       <c r="F346" s="3"/>
@@ -62777,9 +63663,15 @@
       <c r="J346" s="3"/>
     </row>
     <row r="347" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A347" s="8"/>
-      <c r="B347" s="8"/>
-      <c r="C347" s="8"/>
+      <c r="A347" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B347" s="9" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C347" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D347" s="8"/>
       <c r="E347" s="3"/>
       <c r="F347" s="3"/>
@@ -62789,9 +63681,15 @@
       <c r="J347" s="3"/>
     </row>
     <row r="348" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A348" s="8"/>
-      <c r="B348" s="8"/>
-      <c r="C348" s="8"/>
+      <c r="A348" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B348" s="9" t="s">
+        <v>906</v>
+      </c>
+      <c r="C348" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D348" s="8"/>
       <c r="E348" s="3"/>
       <c r="F348" s="3"/>
@@ -62801,9 +63699,15 @@
       <c r="J348" s="3"/>
     </row>
     <row r="349" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A349" s="8"/>
-      <c r="B349" s="8"/>
-      <c r="C349" s="8"/>
+      <c r="A349" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B349" s="9" t="s">
+        <v>1137</v>
+      </c>
+      <c r="C349" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D349" s="8"/>
       <c r="E349" s="3"/>
       <c r="F349" s="3"/>
@@ -62813,9 +63717,15 @@
       <c r="J349" s="3"/>
     </row>
     <row r="350" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A350" s="8"/>
-      <c r="B350" s="8"/>
-      <c r="C350" s="8"/>
+      <c r="A350" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B350" s="9" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C350" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D350" s="8"/>
       <c r="E350" s="3"/>
       <c r="F350" s="3"/>
@@ -62825,9 +63735,15 @@
       <c r="J350" s="3"/>
     </row>
     <row r="351" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A351" s="8"/>
-      <c r="B351" s="8"/>
-      <c r="C351" s="8"/>
+      <c r="A351" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B351" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C351" s="9" t="s">
+        <v>1075</v>
+      </c>
       <c r="D351" s="8"/>
       <c r="E351" s="3"/>
       <c r="F351" s="3"/>
@@ -62837,9 +63753,15 @@
       <c r="J351" s="3"/>
     </row>
     <row r="352" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A352" s="8"/>
-      <c r="B352" s="8"/>
-      <c r="C352" s="8"/>
+      <c r="A352" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B352" s="9" t="s">
+        <v>744</v>
+      </c>
+      <c r="C352" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D352" s="8"/>
       <c r="E352" s="3"/>
       <c r="F352" s="3"/>
@@ -62849,9 +63771,15 @@
       <c r="J352" s="3"/>
     </row>
     <row r="353" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A353" s="8"/>
-      <c r="B353" s="8"/>
-      <c r="C353" s="8"/>
+      <c r="A353" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B353" s="9" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C353" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D353" s="8"/>
       <c r="E353" s="3"/>
       <c r="F353" s="3"/>
@@ -62861,9 +63789,15 @@
       <c r="J353" s="3"/>
     </row>
     <row r="354" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A354" s="8"/>
-      <c r="B354" s="8"/>
-      <c r="C354" s="8"/>
+      <c r="A354" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B354" s="9" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C354" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D354" s="8"/>
       <c r="E354" s="3"/>
       <c r="F354" s="3"/>
@@ -62873,9 +63807,15 @@
       <c r="J354" s="3"/>
     </row>
     <row r="355" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A355" s="8"/>
-      <c r="B355" s="8"/>
-      <c r="C355" s="8"/>
+      <c r="A355" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B355" s="9" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C355" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D355" s="8"/>
       <c r="E355" s="3"/>
       <c r="F355" s="3"/>
@@ -62885,9 +63825,15 @@
       <c r="J355" s="3"/>
     </row>
     <row r="356" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A356" s="8"/>
-      <c r="B356" s="8"/>
-      <c r="C356" s="8"/>
+      <c r="A356" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B356" s="10" t="s">
+        <v>744</v>
+      </c>
+      <c r="C356" s="9" t="s">
+        <v>1066</v>
+      </c>
       <c r="D356" s="8"/>
       <c r="E356" s="3"/>
       <c r="F356" s="3"/>
@@ -62897,9 +63843,15 @@
       <c r="J356" s="3"/>
     </row>
     <row r="357" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A357" s="8"/>
-      <c r="B357" s="8"/>
-      <c r="C357" s="8"/>
+      <c r="A357" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B357" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C357" s="9" t="s">
+        <v>1029</v>
+      </c>
       <c r="D357" s="8"/>
       <c r="E357" s="3"/>
       <c r="F357" s="3"/>
@@ -62909,9 +63861,15 @@
       <c r="J357" s="3"/>
     </row>
     <row r="358" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A358" s="8"/>
-      <c r="B358" s="8"/>
-      <c r="C358" s="8"/>
+      <c r="A358" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B358" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C358" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D358" s="8"/>
       <c r="E358" s="3"/>
       <c r="F358" s="3"/>
@@ -62921,9 +63879,15 @@
       <c r="J358" s="3"/>
     </row>
     <row r="359" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A359" s="8"/>
-      <c r="B359" s="8"/>
-      <c r="C359" s="8"/>
+      <c r="A359" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B359" s="9" t="s">
+        <v>742</v>
+      </c>
+      <c r="C359" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D359" s="8"/>
       <c r="E359" s="3"/>
       <c r="F359" s="3"/>
@@ -62933,9 +63897,15 @@
       <c r="J359" s="3"/>
     </row>
     <row r="360" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A360" s="8"/>
-      <c r="B360" s="8"/>
-      <c r="C360" s="8"/>
+      <c r="A360" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B360" s="9" t="s">
+        <v>741</v>
+      </c>
+      <c r="C360" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D360" s="8"/>
       <c r="E360" s="3"/>
       <c r="F360" s="3"/>
@@ -62945,9 +63915,15 @@
       <c r="J360" s="3"/>
     </row>
     <row r="361" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A361" s="8"/>
-      <c r="B361" s="8"/>
-      <c r="C361" s="8"/>
+      <c r="A361" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B361" s="9" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C361" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D361" s="8"/>
       <c r="E361" s="3"/>
       <c r="F361" s="3"/>
@@ -62957,9 +63933,15 @@
       <c r="J361" s="3"/>
     </row>
     <row r="362" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A362" s="8"/>
-      <c r="B362" s="8"/>
-      <c r="C362" s="8"/>
+      <c r="A362" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B362" s="9" t="s">
+        <v>1142</v>
+      </c>
+      <c r="C362" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D362" s="8"/>
       <c r="E362" s="3"/>
       <c r="F362" s="3"/>
@@ -62969,9 +63951,15 @@
       <c r="J362" s="3"/>
     </row>
     <row r="363" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A363" s="8"/>
-      <c r="B363" s="8"/>
-      <c r="C363" s="8"/>
+      <c r="A363" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B363" s="9" t="s">
+        <v>933</v>
+      </c>
+      <c r="C363" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D363" s="8"/>
       <c r="E363" s="3"/>
       <c r="F363" s="3"/>
@@ -62981,9 +63969,15 @@
       <c r="J363" s="3"/>
     </row>
     <row r="364" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A364" s="8"/>
-      <c r="B364" s="8"/>
-      <c r="C364" s="8"/>
+      <c r="A364" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B364" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C364" s="9" t="s">
+        <v>1061</v>
+      </c>
       <c r="D364" s="8"/>
       <c r="E364" s="3"/>
       <c r="F364" s="3"/>
@@ -62993,9 +63987,15 @@
       <c r="J364" s="3"/>
     </row>
     <row r="365" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A365" s="8"/>
-      <c r="B365" s="8"/>
-      <c r="C365" s="8"/>
+      <c r="A365" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B365" s="9" t="s">
+        <v>1149</v>
+      </c>
+      <c r="C365" s="9" t="s">
+        <v>1048</v>
+      </c>
       <c r="D365" s="8"/>
       <c r="E365" s="3"/>
       <c r="F365" s="3"/>
@@ -63005,9 +64005,15 @@
       <c r="J365" s="3"/>
     </row>
     <row r="366" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A366" s="8"/>
-      <c r="B366" s="8"/>
-      <c r="C366" s="8"/>
+      <c r="A366" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B366" s="9" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C366" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D366" s="8"/>
       <c r="E366" s="3"/>
       <c r="F366" s="3"/>
@@ -63017,9 +64023,15 @@
       <c r="J366" s="3"/>
     </row>
     <row r="367" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A367" s="8"/>
-      <c r="B367" s="8"/>
-      <c r="C367" s="8"/>
+      <c r="A367" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B367" s="9" t="s">
+        <v>1150</v>
+      </c>
+      <c r="C367" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D367" s="8"/>
       <c r="E367" s="3"/>
       <c r="F367" s="3"/>
@@ -63029,9 +64041,15 @@
       <c r="J367" s="3"/>
     </row>
     <row r="368" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A368" s="8"/>
-      <c r="B368" s="8"/>
-      <c r="C368" s="8"/>
+      <c r="A368" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B368" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C368" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D368" s="8"/>
       <c r="E368" s="3"/>
       <c r="F368" s="3"/>
@@ -63041,9 +64059,15 @@
       <c r="J368" s="3"/>
     </row>
     <row r="369" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A369" s="8"/>
-      <c r="B369" s="8"/>
-      <c r="C369" s="8"/>
+      <c r="A369" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B369" s="9" t="s">
+        <v>692</v>
+      </c>
+      <c r="C369" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D369" s="8"/>
       <c r="E369" s="3"/>
       <c r="F369" s="3"/>
@@ -63053,9 +64077,15 @@
       <c r="J369" s="3"/>
     </row>
     <row r="370" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A370" s="8"/>
-      <c r="B370" s="8"/>
-      <c r="C370" s="8"/>
+      <c r="A370" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B370" s="9" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C370" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D370" s="8"/>
       <c r="E370" s="3"/>
       <c r="F370" s="3"/>
@@ -63065,9 +64095,15 @@
       <c r="J370" s="3"/>
     </row>
     <row r="371" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A371" s="8"/>
-      <c r="B371" s="8"/>
-      <c r="C371" s="8"/>
+      <c r="A371" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B371" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="C371" s="9" t="s">
+        <v>1040</v>
+      </c>
       <c r="D371" s="8"/>
       <c r="E371" s="3"/>
       <c r="F371" s="3"/>
@@ -63077,9 +64113,15 @@
       <c r="J371" s="3"/>
     </row>
     <row r="372" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A372" s="8"/>
-      <c r="B372" s="8"/>
-      <c r="C372" s="8"/>
+      <c r="A372" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B372" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="C372" s="9" t="s">
+        <v>1051</v>
+      </c>
       <c r="D372" s="8"/>
       <c r="E372" s="3"/>
       <c r="F372" s="3"/>
@@ -63089,9 +64131,15 @@
       <c r="J372" s="3"/>
     </row>
     <row r="373" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A373" s="8"/>
-      <c r="B373" s="8"/>
-      <c r="C373" s="8"/>
+      <c r="A373" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B373" s="9" t="s">
+        <v>781</v>
+      </c>
+      <c r="C373" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D373" s="8"/>
       <c r="E373" s="3"/>
       <c r="F373" s="3"/>
@@ -63101,9 +64149,15 @@
       <c r="J373" s="3"/>
     </row>
     <row r="374" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A374" s="8"/>
-      <c r="B374" s="8"/>
-      <c r="C374" s="8"/>
+      <c r="A374" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B374" s="10" t="s">
+        <v>744</v>
+      </c>
+      <c r="C374" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D374" s="8"/>
       <c r="E374" s="3"/>
       <c r="F374" s="3"/>
@@ -63113,9 +64167,15 @@
       <c r="J374" s="3"/>
     </row>
     <row r="375" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A375" s="8"/>
-      <c r="B375" s="8"/>
-      <c r="C375" s="8"/>
+      <c r="A375" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B375" s="9" t="s">
+        <v>700</v>
+      </c>
+      <c r="C375" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D375" s="8"/>
       <c r="E375" s="3"/>
       <c r="F375" s="3"/>
@@ -63125,9 +64185,15 @@
       <c r="J375" s="3"/>
     </row>
     <row r="376" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A376" s="8"/>
-      <c r="B376" s="8"/>
-      <c r="C376" s="8"/>
+      <c r="A376" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B376" s="9" t="s">
+        <v>1138</v>
+      </c>
+      <c r="C376" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D376" s="8"/>
       <c r="E376" s="3"/>
       <c r="F376" s="3"/>
@@ -63137,9 +64203,15 @@
       <c r="J376" s="3"/>
     </row>
     <row r="377" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A377" s="8"/>
-      <c r="B377" s="8"/>
-      <c r="C377" s="8"/>
+      <c r="A377" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B377" s="9" t="s">
+        <v>1116</v>
+      </c>
+      <c r="C377" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D377" s="8"/>
       <c r="E377" s="3"/>
       <c r="F377" s="3"/>
@@ -63149,9 +64221,15 @@
       <c r="J377" s="3"/>
     </row>
     <row r="378" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A378" s="8"/>
-      <c r="B378" s="8"/>
-      <c r="C378" s="8"/>
+      <c r="A378" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B378" s="9" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C378" s="9" t="s">
+        <v>1031</v>
+      </c>
       <c r="D378" s="8"/>
       <c r="E378" s="3"/>
       <c r="F378" s="3"/>
@@ -63161,9 +64239,15 @@
       <c r="J378" s="3"/>
     </row>
     <row r="379" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A379" s="8"/>
-      <c r="B379" s="8"/>
-      <c r="C379" s="8"/>
+      <c r="A379" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B379" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C379" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D379" s="8"/>
       <c r="E379" s="3"/>
       <c r="F379" s="3"/>
@@ -63173,9 +64257,15 @@
       <c r="J379" s="3"/>
     </row>
     <row r="380" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A380" s="8"/>
-      <c r="B380" s="8"/>
-      <c r="C380" s="8"/>
+      <c r="A380" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B380" s="9" t="s">
+        <v>768</v>
+      </c>
+      <c r="C380" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D380" s="8"/>
       <c r="E380" s="3"/>
       <c r="F380" s="3"/>
@@ -63185,9 +64275,15 @@
       <c r="J380" s="3"/>
     </row>
     <row r="381" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A381" s="8"/>
-      <c r="B381" s="8"/>
-      <c r="C381" s="8"/>
+      <c r="A381" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B381" s="9" t="s">
+        <v>736</v>
+      </c>
+      <c r="C381" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D381" s="8"/>
       <c r="E381" s="3"/>
       <c r="F381" s="3"/>
@@ -63197,9 +64293,15 @@
       <c r="J381" s="3"/>
     </row>
     <row r="382" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A382" s="8"/>
-      <c r="B382" s="8"/>
-      <c r="C382" s="8"/>
+      <c r="A382" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B382" s="9" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C382" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D382" s="8"/>
       <c r="E382" s="3"/>
       <c r="F382" s="3"/>
@@ -63209,9 +64311,15 @@
       <c r="J382" s="3"/>
     </row>
     <row r="383" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A383" s="8"/>
-      <c r="B383" s="8"/>
-      <c r="C383" s="8"/>
+      <c r="A383" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B383" s="9" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C383" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D383" s="8"/>
       <c r="E383" s="3"/>
       <c r="F383" s="3"/>
@@ -63221,9 +64329,15 @@
       <c r="J383" s="3"/>
     </row>
     <row r="384" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A384" s="8"/>
-      <c r="B384" s="8"/>
-      <c r="C384" s="8"/>
+      <c r="A384" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B384" s="9" t="s">
+        <v>1151</v>
+      </c>
+      <c r="C384" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D384" s="8"/>
       <c r="E384" s="3"/>
       <c r="F384" s="3"/>
@@ -63233,9 +64347,15 @@
       <c r="J384" s="3"/>
     </row>
     <row r="385" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A385" s="8"/>
-      <c r="B385" s="8"/>
-      <c r="C385" s="8"/>
+      <c r="A385" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B385" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C385" s="9" t="s">
+        <v>1066</v>
+      </c>
       <c r="D385" s="8"/>
       <c r="E385" s="3"/>
       <c r="F385" s="3"/>
@@ -63245,9 +64365,15 @@
       <c r="J385" s="3"/>
     </row>
     <row r="386" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A386" s="8"/>
-      <c r="B386" s="8"/>
-      <c r="C386" s="8"/>
+      <c r="A386" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B386" s="9" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C386" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D386" s="8"/>
       <c r="E386" s="3"/>
       <c r="F386" s="3"/>
@@ -63257,9 +64383,15 @@
       <c r="J386" s="3"/>
     </row>
     <row r="387" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A387" s="8"/>
-      <c r="B387" s="8"/>
-      <c r="C387" s="8"/>
+      <c r="A387" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B387" s="9" t="s">
+        <v>1134</v>
+      </c>
+      <c r="C387" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D387" s="8"/>
       <c r="E387" s="3"/>
       <c r="F387" s="3"/>
@@ -63269,9 +64401,15 @@
       <c r="J387" s="3"/>
     </row>
     <row r="388" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A388" s="8"/>
-      <c r="B388" s="8"/>
-      <c r="C388" s="8"/>
+      <c r="A388" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B388" s="9" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C388" s="9" t="s">
+        <v>1040</v>
+      </c>
       <c r="D388" s="8"/>
       <c r="E388" s="3"/>
       <c r="F388" s="3"/>
@@ -63281,9 +64419,15 @@
       <c r="J388" s="3"/>
     </row>
     <row r="389" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A389" s="8"/>
-      <c r="B389" s="8"/>
-      <c r="C389" s="8"/>
+      <c r="A389" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B389" s="9" t="s">
+        <v>1153</v>
+      </c>
+      <c r="C389" s="9" t="s">
+        <v>1040</v>
+      </c>
       <c r="D389" s="8"/>
       <c r="E389" s="3"/>
       <c r="F389" s="3"/>
@@ -63293,9 +64437,15 @@
       <c r="J389" s="3"/>
     </row>
     <row r="390" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A390" s="8"/>
-      <c r="B390" s="8"/>
-      <c r="C390" s="8"/>
+      <c r="A390" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B390" s="9" t="s">
+        <v>766</v>
+      </c>
+      <c r="C390" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D390" s="8"/>
       <c r="E390" s="3"/>
       <c r="F390" s="3"/>
@@ -63305,9 +64455,15 @@
       <c r="J390" s="3"/>
     </row>
     <row r="391" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A391" s="8"/>
-      <c r="B391" s="8"/>
-      <c r="C391" s="8"/>
+      <c r="A391" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B391" s="9" t="s">
+        <v>770</v>
+      </c>
+      <c r="C391" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D391" s="8"/>
       <c r="E391" s="3"/>
       <c r="F391" s="3"/>
@@ -63317,9 +64473,15 @@
       <c r="J391" s="3"/>
     </row>
     <row r="392" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A392" s="8"/>
-      <c r="B392" s="8"/>
-      <c r="C392" s="8"/>
+      <c r="A392" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B392" s="9" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C392" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D392" s="8"/>
       <c r="E392" s="3"/>
       <c r="F392" s="3"/>
@@ -63329,9 +64491,15 @@
       <c r="J392" s="3"/>
     </row>
     <row r="393" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A393" s="8"/>
-      <c r="B393" s="8"/>
-      <c r="C393" s="8"/>
+      <c r="A393" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B393" s="9" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C393" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D393" s="8"/>
       <c r="E393" s="3"/>
       <c r="F393" s="3"/>
@@ -63341,9 +64509,15 @@
       <c r="J393" s="3"/>
     </row>
     <row r="394" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A394" s="8"/>
-      <c r="B394" s="8"/>
-      <c r="C394" s="8"/>
+      <c r="A394" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B394" s="9" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C394" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D394" s="8"/>
       <c r="E394" s="3"/>
       <c r="F394" s="3"/>
@@ -63353,9 +64527,15 @@
       <c r="J394" s="3"/>
     </row>
     <row r="395" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A395" s="8"/>
-      <c r="B395" s="8"/>
-      <c r="C395" s="8"/>
+      <c r="A395" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B395" s="9" t="s">
+        <v>1147</v>
+      </c>
+      <c r="C395" s="9" t="s">
+        <v>1043</v>
+      </c>
       <c r="D395" s="8"/>
       <c r="E395" s="3"/>
       <c r="F395" s="3"/>
@@ -63365,9 +64545,15 @@
       <c r="J395" s="3"/>
     </row>
     <row r="396" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A396" s="8"/>
-      <c r="B396" s="8"/>
-      <c r="C396" s="8"/>
+      <c r="A396" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B396" s="9" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C396" s="10" t="s">
+        <v>1039</v>
+      </c>
       <c r="D396" s="8"/>
       <c r="E396" s="3"/>
       <c r="F396" s="3"/>
@@ -63377,9 +64563,15 @@
       <c r="J396" s="3"/>
     </row>
     <row r="397" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A397" s="8"/>
-      <c r="B397" s="8"/>
-      <c r="C397" s="8"/>
+      <c r="A397" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B397" s="9" t="s">
+        <v>959</v>
+      </c>
+      <c r="C397" s="9" t="s">
+        <v>1033</v>
+      </c>
       <c r="D397" s="8"/>
       <c r="E397" s="3"/>
       <c r="F397" s="3"/>
@@ -63389,9 +64581,15 @@
       <c r="J397" s="3"/>
     </row>
     <row r="398" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A398" s="8"/>
-      <c r="B398" s="8"/>
-      <c r="C398" s="8"/>
+      <c r="A398" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B398" s="9" t="s">
+        <v>1155</v>
+      </c>
+      <c r="C398" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D398" s="8"/>
       <c r="E398" s="3"/>
       <c r="F398" s="3"/>
@@ -63401,9 +64599,15 @@
       <c r="J398" s="3"/>
     </row>
     <row r="399" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A399" s="8"/>
-      <c r="B399" s="8"/>
-      <c r="C399" s="8"/>
+      <c r="A399" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B399" s="9" t="s">
+        <v>773</v>
+      </c>
+      <c r="C399" s="9" t="s">
+        <v>1070</v>
+      </c>
       <c r="D399" s="8"/>
       <c r="E399" s="3"/>
       <c r="F399" s="3"/>
@@ -63413,9 +64617,15 @@
       <c r="J399" s="3"/>
     </row>
     <row r="400" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A400" s="8"/>
-      <c r="B400" s="8"/>
-      <c r="C400" s="8"/>
+      <c r="A400" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B400" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C400" s="9" t="s">
+        <v>1070</v>
+      </c>
       <c r="D400" s="8"/>
       <c r="E400" s="3"/>
       <c r="F400" s="3"/>
@@ -63425,9 +64635,15 @@
       <c r="J400" s="3"/>
     </row>
     <row r="401" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A401" s="8"/>
-      <c r="B401" s="8"/>
-      <c r="C401" s="8"/>
+      <c r="A401" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B401" s="9" t="s">
+        <v>1143</v>
+      </c>
+      <c r="C401" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D401" s="8"/>
       <c r="E401" s="3"/>
       <c r="F401" s="3"/>
@@ -63437,9 +64653,15 @@
       <c r="J401" s="3"/>
     </row>
     <row r="402" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A402" s="8"/>
-      <c r="B402" s="8"/>
-      <c r="C402" s="8"/>
+      <c r="A402" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B402" s="9" t="s">
+        <v>1125</v>
+      </c>
+      <c r="C402" s="10" t="s">
+        <v>1047</v>
+      </c>
       <c r="D402" s="8"/>
       <c r="E402" s="3"/>
       <c r="F402" s="3"/>
@@ -63449,9 +64671,15 @@
       <c r="J402" s="3"/>
     </row>
     <row r="403" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A403" s="8"/>
-      <c r="B403" s="8"/>
-      <c r="C403" s="8"/>
+      <c r="A403" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B403" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C403" s="9" t="s">
+        <v>1048</v>
+      </c>
       <c r="D403" s="8"/>
       <c r="E403" s="3"/>
       <c r="F403" s="3"/>
@@ -63461,9 +64689,15 @@
       <c r="J403" s="3"/>
     </row>
     <row r="404" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A404" s="8"/>
-      <c r="B404" s="8"/>
-      <c r="C404" s="8"/>
+      <c r="A404" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B404" s="9" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C404" s="9" t="s">
+        <v>1048</v>
+      </c>
       <c r="D404" s="8"/>
       <c r="E404" s="3"/>
       <c r="F404" s="3"/>
@@ -63473,9 +64707,15 @@
       <c r="J404" s="3"/>
     </row>
     <row r="405" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A405" s="8"/>
-      <c r="B405" s="8"/>
-      <c r="C405" s="8"/>
+      <c r="A405" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B405" s="10" t="s">
+        <v>959</v>
+      </c>
+      <c r="C405" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D405" s="8"/>
       <c r="E405" s="3"/>
       <c r="F405" s="3"/>
@@ -63485,9 +64725,15 @@
       <c r="J405" s="3"/>
     </row>
     <row r="406" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A406" s="8"/>
-      <c r="B406" s="8"/>
-      <c r="C406" s="8"/>
+      <c r="A406" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B406" s="9" t="s">
+        <v>933</v>
+      </c>
+      <c r="C406" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D406" s="8"/>
       <c r="E406" s="3"/>
       <c r="F406" s="3"/>
@@ -63497,9 +64743,15 @@
       <c r="J406" s="3"/>
     </row>
     <row r="407" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A407" s="8"/>
-      <c r="B407" s="8"/>
-      <c r="C407" s="8"/>
+      <c r="A407" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B407" s="9" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C407" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D407" s="8"/>
       <c r="E407" s="3"/>
       <c r="F407" s="3"/>
@@ -63509,9 +64761,15 @@
       <c r="J407" s="3"/>
     </row>
     <row r="408" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A408" s="8"/>
-      <c r="B408" s="8"/>
-      <c r="C408" s="8"/>
+      <c r="A408" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B408" s="9" t="s">
+        <v>761</v>
+      </c>
+      <c r="C408" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D408" s="8"/>
       <c r="E408" s="3"/>
       <c r="F408" s="3"/>
@@ -63521,9 +64779,15 @@
       <c r="J408" s="3"/>
     </row>
     <row r="409" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A409" s="8"/>
-      <c r="B409" s="8"/>
-      <c r="C409" s="8"/>
+      <c r="A409" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B409" s="9" t="s">
+        <v>1128</v>
+      </c>
+      <c r="C409" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D409" s="8"/>
       <c r="E409" s="3"/>
       <c r="F409" s="3"/>
@@ -63533,9 +64797,15 @@
       <c r="J409" s="3"/>
     </row>
     <row r="410" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A410" s="8"/>
-      <c r="B410" s="8"/>
-      <c r="C410" s="8"/>
+      <c r="A410" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B410" s="9" t="s">
+        <v>755</v>
+      </c>
+      <c r="C410" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D410" s="8"/>
       <c r="E410" s="3"/>
       <c r="F410" s="3"/>
@@ -63545,9 +64815,15 @@
       <c r="J410" s="3"/>
     </row>
     <row r="411" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A411" s="8"/>
-      <c r="B411" s="8"/>
-      <c r="C411" s="8"/>
+      <c r="A411" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B411" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C411" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D411" s="8"/>
       <c r="E411" s="3"/>
       <c r="F411" s="3"/>
@@ -63557,9 +64833,15 @@
       <c r="J411" s="3"/>
     </row>
     <row r="412" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A412" s="8"/>
-      <c r="B412" s="8"/>
-      <c r="C412" s="8"/>
+      <c r="A412" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B412" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C412" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D412" s="8"/>
       <c r="E412" s="3"/>
       <c r="F412" s="3"/>
@@ -63569,9 +64851,15 @@
       <c r="J412" s="3"/>
     </row>
     <row r="413" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A413" s="8"/>
-      <c r="B413" s="8"/>
-      <c r="C413" s="8"/>
+      <c r="A413" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B413" s="9" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C413" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D413" s="8"/>
       <c r="E413" s="3"/>
       <c r="F413" s="3"/>
@@ -63581,9 +64869,15 @@
       <c r="J413" s="3"/>
     </row>
     <row r="414" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A414" s="8"/>
-      <c r="B414" s="8"/>
-      <c r="C414" s="8"/>
+      <c r="A414" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B414" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C414" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D414" s="8"/>
       <c r="E414" s="3"/>
       <c r="F414" s="3"/>
@@ -63593,9 +64887,15 @@
       <c r="J414" s="3"/>
     </row>
     <row r="415" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A415" s="8"/>
-      <c r="B415" s="8"/>
-      <c r="C415" s="8"/>
+      <c r="A415" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B415" s="9" t="s">
+        <v>933</v>
+      </c>
+      <c r="C415" s="9" t="s">
+        <v>1048</v>
+      </c>
       <c r="D415" s="8"/>
       <c r="E415" s="3"/>
       <c r="F415" s="3"/>
@@ -63605,9 +64905,15 @@
       <c r="J415" s="3"/>
     </row>
     <row r="416" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A416" s="8"/>
-      <c r="B416" s="8"/>
-      <c r="C416" s="8"/>
+      <c r="A416" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B416" s="9" t="s">
+        <v>755</v>
+      </c>
+      <c r="C416" s="9" t="s">
+        <v>1066</v>
+      </c>
       <c r="D416" s="8"/>
       <c r="E416" s="3"/>
       <c r="F416" s="3"/>
@@ -63617,9 +64923,15 @@
       <c r="J416" s="3"/>
     </row>
     <row r="417" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A417" s="8"/>
-      <c r="B417" s="8"/>
-      <c r="C417" s="8"/>
+      <c r="A417" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B417" s="9" t="s">
+        <v>880</v>
+      </c>
+      <c r="C417" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D417" s="8"/>
       <c r="E417" s="3"/>
       <c r="F417" s="3"/>
@@ -63629,9 +64941,15 @@
       <c r="J417" s="3"/>
     </row>
     <row r="418" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A418" s="8"/>
-      <c r="B418" s="8"/>
-      <c r="C418" s="8"/>
+      <c r="A418" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B418" s="9" t="s">
+        <v>767</v>
+      </c>
+      <c r="C418" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D418" s="8"/>
       <c r="E418" s="3"/>
       <c r="F418" s="3"/>
@@ -63641,9 +64959,15 @@
       <c r="J418" s="3"/>
     </row>
     <row r="419" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A419" s="8"/>
-      <c r="B419" s="8"/>
-      <c r="C419" s="8"/>
+      <c r="A419" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B419" s="9" t="s">
+        <v>1139</v>
+      </c>
+      <c r="C419" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D419" s="8"/>
       <c r="E419" s="3"/>
       <c r="F419" s="3"/>
@@ -63653,9 +64977,15 @@
       <c r="J419" s="3"/>
     </row>
     <row r="420" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A420" s="8"/>
-      <c r="B420" s="8"/>
-      <c r="C420" s="8"/>
+      <c r="A420" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B420" s="9" t="s">
+        <v>1157</v>
+      </c>
+      <c r="C420" s="9" t="s">
+        <v>1077</v>
+      </c>
       <c r="D420" s="8"/>
       <c r="E420" s="3"/>
       <c r="F420" s="3"/>
@@ -63665,9 +64995,15 @@
       <c r="J420" s="3"/>
     </row>
     <row r="421" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A421" s="8"/>
-      <c r="B421" s="8"/>
-      <c r="C421" s="8"/>
+      <c r="A421" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B421" s="9" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C421" s="9" t="s">
+        <v>1076</v>
+      </c>
       <c r="D421" s="8"/>
       <c r="E421" s="3"/>
       <c r="F421" s="3"/>
@@ -63677,9 +65013,15 @@
       <c r="J421" s="3"/>
     </row>
     <row r="422" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A422" s="8"/>
-      <c r="B422" s="8"/>
-      <c r="C422" s="8"/>
+      <c r="A422" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B422" s="9" t="s">
+        <v>692</v>
+      </c>
+      <c r="C422" s="9" t="s">
+        <v>1030</v>
+      </c>
       <c r="D422" s="8"/>
       <c r="E422" s="3"/>
       <c r="F422" s="3"/>
@@ -63689,9 +65031,15 @@
       <c r="J422" s="3"/>
     </row>
     <row r="423" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A423" s="8"/>
-      <c r="B423" s="8"/>
-      <c r="C423" s="8"/>
+      <c r="A423" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B423" s="9" t="s">
+        <v>743</v>
+      </c>
+      <c r="C423" s="9" t="s">
+        <v>1047</v>
+      </c>
       <c r="D423" s="8"/>
       <c r="E423" s="3"/>
       <c r="F423" s="3"/>
@@ -63701,9 +65049,15 @@
       <c r="J423" s="3"/>
     </row>
     <row r="424" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A424" s="8"/>
-      <c r="B424" s="8"/>
-      <c r="C424" s="8"/>
+      <c r="A424" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B424" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C424" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D424" s="8"/>
       <c r="E424" s="3"/>
       <c r="F424" s="3"/>
@@ -63713,9 +65067,15 @@
       <c r="J424" s="3"/>
     </row>
     <row r="425" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A425" s="8"/>
-      <c r="B425" s="8"/>
-      <c r="C425" s="8"/>
+      <c r="A425" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B425" s="10" t="s">
+        <v>967</v>
+      </c>
+      <c r="C425" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D425" s="8"/>
       <c r="E425" s="3"/>
       <c r="F425" s="3"/>
@@ -63725,9 +65085,15 @@
       <c r="J425" s="3"/>
     </row>
     <row r="426" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A426" s="8"/>
-      <c r="B426" s="8"/>
-      <c r="C426" s="8"/>
+      <c r="A426" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B426" s="9" t="s">
+        <v>1118</v>
+      </c>
+      <c r="C426" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D426" s="8"/>
       <c r="E426" s="3"/>
       <c r="F426" s="3"/>
@@ -63737,9 +65103,15 @@
       <c r="J426" s="3"/>
     </row>
     <row r="427" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A427" s="8"/>
-      <c r="B427" s="8"/>
-      <c r="C427" s="8"/>
+      <c r="A427" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B427" s="9" t="s">
+        <v>967</v>
+      </c>
+      <c r="C427" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D427" s="8"/>
       <c r="E427" s="3"/>
       <c r="F427" s="3"/>
@@ -63749,9 +65121,15 @@
       <c r="J427" s="3"/>
     </row>
     <row r="428" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A428" s="8"/>
-      <c r="B428" s="8"/>
-      <c r="C428" s="8"/>
+      <c r="A428" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B428" s="9" t="s">
+        <v>902</v>
+      </c>
+      <c r="C428" s="9" t="s">
+        <v>1032</v>
+      </c>
       <c r="D428" s="8"/>
       <c r="E428" s="3"/>
       <c r="F428" s="3"/>
@@ -63761,9 +65139,15 @@
       <c r="J428" s="3"/>
     </row>
     <row r="429" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A429" s="8"/>
-      <c r="B429" s="8"/>
-      <c r="C429" s="8"/>
+      <c r="A429" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B429" s="9" t="s">
+        <v>736</v>
+      </c>
+      <c r="C429" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D429" s="8"/>
       <c r="E429" s="3"/>
       <c r="F429" s="3"/>
@@ -63773,9 +65157,15 @@
       <c r="J429" s="3"/>
     </row>
     <row r="430" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A430" s="8"/>
-      <c r="B430" s="8"/>
-      <c r="C430" s="8"/>
+      <c r="A430" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B430" s="9" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C430" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D430" s="8"/>
       <c r="E430" s="3"/>
       <c r="F430" s="3"/>
@@ -63785,9 +65175,15 @@
       <c r="J430" s="3"/>
     </row>
     <row r="431" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A431" s="8"/>
-      <c r="B431" s="8"/>
-      <c r="C431" s="8"/>
+      <c r="A431" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B431" s="9" t="s">
+        <v>758</v>
+      </c>
+      <c r="C431" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D431" s="8"/>
       <c r="E431" s="3"/>
       <c r="F431" s="3"/>
@@ -63797,9 +65193,15 @@
       <c r="J431" s="3"/>
     </row>
     <row r="432" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A432" s="8"/>
-      <c r="B432" s="8"/>
-      <c r="C432" s="8"/>
+      <c r="A432" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B432" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="C432" s="9" t="s">
+        <v>1042</v>
+      </c>
       <c r="D432" s="8"/>
       <c r="E432" s="3"/>
       <c r="F432" s="3"/>
@@ -63809,9 +65211,15 @@
       <c r="J432" s="3"/>
     </row>
     <row r="433" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A433" s="8"/>
-      <c r="B433" s="8"/>
-      <c r="C433" s="8"/>
+      <c r="A433" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B433" s="9" t="s">
+        <v>1154</v>
+      </c>
+      <c r="C433" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D433" s="8"/>
       <c r="E433" s="3"/>
       <c r="F433" s="3"/>
@@ -63821,9 +65229,15 @@
       <c r="J433" s="3"/>
     </row>
     <row r="434" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A434" s="8"/>
-      <c r="B434" s="8"/>
-      <c r="C434" s="8"/>
+      <c r="A434" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B434" s="9" t="s">
+        <v>748</v>
+      </c>
+      <c r="C434" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D434" s="8"/>
       <c r="E434" s="3"/>
       <c r="F434" s="3"/>
@@ -63833,9 +65247,15 @@
       <c r="J434" s="3"/>
     </row>
     <row r="435" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A435" s="8"/>
-      <c r="B435" s="8"/>
-      <c r="C435" s="8"/>
+      <c r="A435" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B435" s="9" t="s">
+        <v>1158</v>
+      </c>
+      <c r="C435" s="9" t="s">
+        <v>1099</v>
+      </c>
       <c r="D435" s="8"/>
       <c r="E435" s="3"/>
       <c r="F435" s="3"/>
@@ -63845,9 +65265,15 @@
       <c r="J435" s="3"/>
     </row>
     <row r="436" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A436" s="8"/>
-      <c r="B436" s="8"/>
-      <c r="C436" s="8"/>
+      <c r="A436" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B436" s="9" t="s">
+        <v>1141</v>
+      </c>
+      <c r="C436" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D436" s="8"/>
       <c r="E436" s="3"/>
       <c r="F436" s="3"/>
@@ -63857,9 +65283,15 @@
       <c r="J436" s="3"/>
     </row>
     <row r="437" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A437" s="8"/>
-      <c r="B437" s="8"/>
-      <c r="C437" s="8"/>
+      <c r="A437" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B437" s="9" t="s">
+        <v>1111</v>
+      </c>
+      <c r="C437" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D437" s="8"/>
       <c r="E437" s="3"/>
       <c r="F437" s="3"/>
@@ -63869,9 +65301,15 @@
       <c r="J437" s="3"/>
     </row>
     <row r="438" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A438" s="8"/>
-      <c r="B438" s="8"/>
-      <c r="C438" s="8"/>
+      <c r="A438" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B438" s="9" t="s">
+        <v>1144</v>
+      </c>
+      <c r="C438" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D438" s="8"/>
       <c r="E438" s="3"/>
       <c r="F438" s="3"/>
@@ -63881,9 +65319,15 @@
       <c r="J438" s="3"/>
     </row>
     <row r="439" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A439" s="8"/>
-      <c r="B439" s="8"/>
-      <c r="C439" s="8"/>
+      <c r="A439" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B439" s="9" t="s">
+        <v>771</v>
+      </c>
+      <c r="C439" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D439" s="8"/>
       <c r="E439" s="3"/>
       <c r="F439" s="3"/>
@@ -63893,9 +65337,15 @@
       <c r="J439" s="3"/>
     </row>
     <row r="440" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A440" s="8"/>
-      <c r="B440" s="8"/>
-      <c r="C440" s="8"/>
+      <c r="A440" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B440" s="9" t="s">
+        <v>741</v>
+      </c>
+      <c r="C440" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D440" s="8"/>
       <c r="E440" s="3"/>
       <c r="F440" s="3"/>
@@ -63905,9 +65355,15 @@
       <c r="J440" s="3"/>
     </row>
     <row r="441" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A441" s="8"/>
-      <c r="B441" s="8"/>
-      <c r="C441" s="8"/>
+      <c r="A441" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B441" s="9" t="s">
+        <v>740</v>
+      </c>
+      <c r="C441" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D441" s="8"/>
       <c r="E441" s="3"/>
       <c r="F441" s="3"/>
@@ -63917,9 +65373,15 @@
       <c r="J441" s="3"/>
     </row>
     <row r="442" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A442" s="8"/>
-      <c r="B442" s="8"/>
-      <c r="C442" s="8"/>
+      <c r="A442" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B442" s="9" t="s">
+        <v>773</v>
+      </c>
+      <c r="C442" s="9" t="s">
+        <v>1075</v>
+      </c>
       <c r="D442" s="8"/>
       <c r="E442" s="3"/>
       <c r="F442" s="3"/>
@@ -63929,9 +65391,15 @@
       <c r="J442" s="3"/>
     </row>
     <row r="443" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A443" s="8"/>
-      <c r="B443" s="8"/>
-      <c r="C443" s="8"/>
+      <c r="A443" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B443" s="9" t="s">
+        <v>707</v>
+      </c>
+      <c r="C443" s="9" t="s">
+        <v>1069</v>
+      </c>
       <c r="D443" s="8"/>
       <c r="E443" s="3"/>
       <c r="F443" s="3"/>
@@ -63941,9 +65409,15 @@
       <c r="J443" s="3"/>
     </row>
     <row r="444" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A444" s="8"/>
-      <c r="B444" s="8"/>
-      <c r="C444" s="8"/>
+      <c r="A444" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B444" s="9" t="s">
+        <v>1159</v>
+      </c>
+      <c r="C444" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D444" s="8"/>
       <c r="E444" s="3"/>
       <c r="F444" s="3"/>
@@ -63953,9 +65427,15 @@
       <c r="J444" s="3"/>
     </row>
     <row r="445" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A445" s="8"/>
-      <c r="B445" s="8"/>
-      <c r="C445" s="8"/>
+      <c r="A445" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B445" s="9" t="s">
+        <v>1152</v>
+      </c>
+      <c r="C445" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D445" s="8"/>
       <c r="E445" s="3"/>
       <c r="F445" s="3"/>
@@ -63965,9 +65445,15 @@
       <c r="J445" s="3"/>
     </row>
     <row r="446" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A446" s="8"/>
-      <c r="B446" s="8"/>
-      <c r="C446" s="8"/>
+      <c r="A446" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B446" s="9" t="s">
+        <v>1156</v>
+      </c>
+      <c r="C446" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D446" s="8"/>
       <c r="E446" s="3"/>
       <c r="F446" s="3"/>
@@ -63977,9 +65463,15 @@
       <c r="J446" s="3"/>
     </row>
     <row r="447" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A447" s="8"/>
-      <c r="B447" s="8"/>
-      <c r="C447" s="8"/>
+      <c r="A447" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B447" s="9" t="s">
+        <v>750</v>
+      </c>
+      <c r="C447" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D447" s="8"/>
       <c r="E447" s="3"/>
       <c r="F447" s="3"/>
@@ -63989,9 +65481,15 @@
       <c r="J447" s="3"/>
     </row>
     <row r="448" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A448" s="8"/>
-      <c r="B448" s="8"/>
-      <c r="C448" s="8"/>
+      <c r="A448" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B448" s="9" t="s">
+        <v>1123</v>
+      </c>
+      <c r="C448" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D448" s="8"/>
       <c r="E448" s="3"/>
       <c r="F448" s="3"/>
@@ -64001,9 +65499,15 @@
       <c r="J448" s="3"/>
     </row>
     <row r="449" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A449" s="8"/>
-      <c r="B449" s="8"/>
-      <c r="C449" s="8"/>
+      <c r="A449" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B449" s="9" t="s">
+        <v>1114</v>
+      </c>
+      <c r="C449" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D449" s="8"/>
       <c r="E449" s="3"/>
       <c r="F449" s="3"/>
@@ -64013,9 +65517,15 @@
       <c r="J449" s="3"/>
     </row>
     <row r="450" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A450" s="8"/>
-      <c r="B450" s="8"/>
-      <c r="C450" s="8"/>
+      <c r="A450" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B450" s="9" t="s">
+        <v>768</v>
+      </c>
+      <c r="C450" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D450" s="8"/>
       <c r="E450" s="3"/>
       <c r="F450" s="3"/>
@@ -64025,9 +65535,15 @@
       <c r="J450" s="3"/>
     </row>
     <row r="451" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A451" s="8"/>
-      <c r="B451" s="8"/>
-      <c r="C451" s="8"/>
+      <c r="A451" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B451" s="9" t="s">
+        <v>1140</v>
+      </c>
+      <c r="C451" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D451" s="8"/>
       <c r="E451" s="3"/>
       <c r="F451" s="3"/>
@@ -64037,9 +65553,15 @@
       <c r="J451" s="3"/>
     </row>
     <row r="452" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A452" s="8"/>
-      <c r="B452" s="8"/>
-      <c r="C452" s="8"/>
+      <c r="A452" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B452" s="9" t="s">
+        <v>761</v>
+      </c>
+      <c r="C452" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D452" s="8"/>
       <c r="E452" s="3"/>
       <c r="F452" s="3"/>
@@ -64049,9 +65571,15 @@
       <c r="J452" s="3"/>
     </row>
     <row r="453" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A453" s="8"/>
-      <c r="B453" s="8"/>
-      <c r="C453" s="8"/>
+      <c r="A453" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B453" s="9" t="s">
+        <v>1145</v>
+      </c>
+      <c r="C453" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D453" s="8"/>
       <c r="E453" s="3"/>
       <c r="F453" s="3"/>
@@ -64061,9 +65589,15 @@
       <c r="J453" s="3"/>
     </row>
     <row r="454" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A454" s="8"/>
-      <c r="B454" s="8"/>
-      <c r="C454" s="8"/>
+      <c r="A454" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B454" s="9" t="s">
+        <v>1146</v>
+      </c>
+      <c r="C454" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D454" s="8"/>
       <c r="E454" s="3"/>
       <c r="F454" s="3"/>
@@ -64073,9 +65607,15 @@
       <c r="J454" s="3"/>
     </row>
     <row r="455" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A455" s="8"/>
-      <c r="B455" s="8"/>
-      <c r="C455" s="8"/>
+      <c r="A455" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B455" s="9" t="s">
+        <v>1127</v>
+      </c>
+      <c r="C455" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D455" s="8"/>
       <c r="E455" s="3"/>
       <c r="F455" s="3"/>
@@ -64085,9 +65625,15 @@
       <c r="J455" s="3"/>
     </row>
     <row r="456" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A456" s="8"/>
-      <c r="B456" s="8"/>
-      <c r="C456" s="8"/>
+      <c r="A456" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B456" s="9" t="s">
+        <v>959</v>
+      </c>
+      <c r="C456" s="9" t="s">
+        <v>1046</v>
+      </c>
       <c r="D456" s="8"/>
       <c r="E456" s="3"/>
       <c r="F456" s="3"/>
@@ -64097,9 +65643,15 @@
       <c r="J456" s="3"/>
     </row>
     <row r="457" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A457" s="8"/>
-      <c r="B457" s="8"/>
-      <c r="C457" s="8"/>
+      <c r="A457" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B457" s="9" t="s">
+        <v>756</v>
+      </c>
+      <c r="C457" s="9" t="s">
+        <v>1107</v>
+      </c>
       <c r="D457" s="8"/>
       <c r="E457" s="3"/>
       <c r="F457" s="3"/>
@@ -64109,9 +65661,15 @@
       <c r="J457" s="3"/>
     </row>
     <row r="458" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A458" s="8"/>
-      <c r="B458" s="8"/>
-      <c r="C458" s="8"/>
+      <c r="A458" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B458" s="9" t="s">
+        <v>1119</v>
+      </c>
+      <c r="C458" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D458" s="8"/>
       <c r="E458" s="3"/>
       <c r="F458" s="3"/>
@@ -64121,9 +65679,15 @@
       <c r="J458" s="3"/>
     </row>
     <row r="459" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A459" s="8"/>
-      <c r="B459" s="8"/>
-      <c r="C459" s="8"/>
+      <c r="A459" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B459" s="9" t="s">
+        <v>1148</v>
+      </c>
+      <c r="C459" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D459" s="8"/>
       <c r="E459" s="3"/>
       <c r="F459" s="3"/>
@@ -64133,9 +65697,15 @@
       <c r="J459" s="3"/>
     </row>
     <row r="460" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A460" s="8"/>
-      <c r="B460" s="8"/>
-      <c r="C460" s="8"/>
+      <c r="A460" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B460" s="9" t="s">
+        <v>765</v>
+      </c>
+      <c r="C460" s="9" t="s">
+        <v>1039</v>
+      </c>
       <c r="D460" s="8"/>
       <c r="E460" s="3"/>
       <c r="F460" s="3"/>
@@ -64145,9 +65715,15 @@
       <c r="J460" s="3"/>
     </row>
     <row r="461" spans="1:10" ht="22.5" customHeight="1">
-      <c r="A461" s="8"/>
-      <c r="B461" s="8"/>
-      <c r="C461" s="8"/>
+      <c r="A461" s="10" t="s">
+        <v>739</v>
+      </c>
+      <c r="B461" s="9" t="s">
+        <v>959</v>
+      </c>
+      <c r="C461" s="9" t="s">
+        <v>1057</v>
+      </c>
       <c r="D461" s="8"/>
       <c r="E461" s="3"/>
       <c r="F461" s="3"/>

</xml_diff>